<commit_message>
projeto antes do teste
vou testar github
</commit_message>
<xml_diff>
--- a/Pasta1project.xlsx
+++ b/Pasta1project.xlsx
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>adawda</t>
         </is>
       </c>
       <c r="C10" s="2" t="n"/>
@@ -1749,8 +1749,10 @@
       <c r="L37" s="6" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="12" t="n">
-        <v>0</v>
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>Felipe</t>
+        </is>
       </c>
       <c r="B38" s="12" t="n">
         <v>1</v>
@@ -1767,8 +1769,10 @@
       <c r="L38" s="6" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="12" t="n">
-        <v>0</v>
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Matheus</t>
+        </is>
       </c>
       <c r="B39" s="12" t="n">
         <v>3</v>
@@ -1785,8 +1789,10 @@
       <c r="L39" s="6" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="12" t="n">
-        <v>0</v>
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Joao</t>
+        </is>
       </c>
       <c r="B40" s="12" t="n">
         <v>3</v>
@@ -1803,8 +1809,10 @@
       <c r="L40" s="6" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="12" t="n">
-        <v>0</v>
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
       </c>
       <c r="B41" s="12" t="n">
         <v>3</v>
@@ -1821,8 +1829,10 @@
       <c r="L41" s="6" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="12" t="n">
-        <v>0</v>
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>Pedro</t>
+        </is>
       </c>
       <c r="B42" s="12" t="n">
         <v>3</v>
@@ -1839,8 +1849,10 @@
       <c r="L42" s="6" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="12" t="n">
-        <v>0</v>
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Andre</t>
+        </is>
       </c>
       <c r="B43" s="12" t="n">
         <v>7</v>
@@ -1857,8 +1869,10 @@
       <c r="L43" s="6" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="12" t="n">
-        <v>0</v>
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>Davi</t>
+        </is>
       </c>
       <c r="B44" s="12" t="n">
         <v>7</v>

</xml_diff>